<commit_message>
bug fixes for telem, move circuits, and load parameters. code structure updates
</commit_message>
<xml_diff>
--- a/CED ElecTools.extension/AE pyTools.tab/Electrical.panel/Circuits1.stack/Circuit Tools.pulldown/Load Electrical Parameters.pushbutton/Content/ELEC SHARED PARAM TABLE.xlsx
+++ b/CED ElecTools.extension/AE pyTools.tab/Electrical.panel/Circuits1.stack/Circuit Tools.pulldown/Load Electrical Parameters.pushbutton/Content/ELEC SHARED PARAM TABLE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aevelina\CED_Extensions\AE pyTools.extension\AE pyTools.Tab\Electrical.panel\Circuits1.stack\Circuit Tools.pulldown\Load Electrical Parameters.pushbutton\Content\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aevelina\CED_Extensions\CED ElecTools.extension\AE pyTools.tab\Electrical.panel\Circuits1.stack\Circuit Tools.pulldown\Load Electrical Parameters.pushbutton\Content\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE4DF8C-E0F0-4EC8-ACC9-CBC5520A00B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{524BA5B9-4421-48FF-B3F1-FC7595F9A471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21855" yWindow="1710" windowWidth="29445" windowHeight="17685" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Parameter List" sheetId="1" r:id="rId1"/>
@@ -109,9 +109,6 @@
     <t>Electrical - Circuiting</t>
   </si>
   <si>
-    <t>Electrical Circuits, Electrical Equipment, Electrical Fixtures</t>
-  </si>
-  <si>
     <t>5bf6a78d-f8b5-4a55-b18f-55dfdf3a8900</t>
   </si>
   <si>
@@ -1505,6 +1502,9 @@
   </si>
   <si>
     <t>Circuit Data_CED</t>
+  </si>
+  <si>
+    <t>All Electrical</t>
   </si>
 </sst>
 </file>
@@ -1931,10 +1931,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>430</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>431</v>
       </c>
       <c r="F1" s="5" t="s">
         <v>3</v>
@@ -1951,13 +1951,13 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
       <c r="B2" s="7">
         <v>1</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>17</v>
@@ -1972,27 +1972,27 @@
         <v>10</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B3" s="7">
         <v>2</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>19</v>
@@ -2001,27 +2001,27 @@
         <v>10</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
       <c r="B4" s="7">
         <v>3</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>19</v>
@@ -2030,27 +2030,27 @@
         <v>10</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
       <c r="B5" s="7">
         <v>4</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>19</v>
@@ -2059,21 +2059,21 @@
         <v>10</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" s="7">
         <v>5</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>17</v>
@@ -2088,10 +2088,10 @@
         <v>10</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -2117,21 +2117,21 @@
         <v>10</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B8" s="7">
         <v>7</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>17</v>
@@ -2146,27 +2146,27 @@
         <v>10</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B9" s="7">
         <v>8</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>19</v>
@@ -2175,27 +2175,27 @@
         <v>10</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" s="7">
         <v>9</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>8</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>19</v>
@@ -2204,21 +2204,21 @@
         <v>10</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" s="7">
         <v>10</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>17</v>
@@ -2233,27 +2233,27 @@
         <v>10</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
       <c r="B12" s="7">
         <v>11</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>19</v>
@@ -2262,27 +2262,27 @@
         <v>10</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="B13" s="7">
         <v>12</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F13" s="1" t="s">
         <v>19</v>
@@ -2290,28 +2290,28 @@
       <c r="G13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>20</v>
+      <c r="H13" s="3" t="s">
+        <v>485</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="B14" s="7">
         <v>13</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F14" s="1" t="s">
         <v>19</v>
@@ -2319,22 +2319,22 @@
       <c r="G14" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>20</v>
+      <c r="H14" s="3" t="s">
+        <v>485</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="B15" s="7">
         <v>14</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>17</v>
@@ -2349,21 +2349,21 @@
         <v>10</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
       <c r="B16" s="7">
         <v>15</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
       <c r="D16" s="4" t="s">
         <v>17</v>
@@ -2378,21 +2378,21 @@
         <v>10</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
       <c r="B17" s="7">
         <v>16</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
       <c r="D17" s="4" t="s">
         <v>17</v>
@@ -2407,27 +2407,27 @@
         <v>10</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B18" s="7">
         <v>17</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="D18" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F18" s="1" t="s">
         <v>19</v>
@@ -2436,27 +2436,27 @@
         <v>10</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B19" s="7">
         <v>18</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F19" s="1" t="s">
         <v>19</v>
@@ -2465,27 +2465,27 @@
         <v>10</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B20" s="7">
         <v>19</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="D20" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>19</v>
@@ -2494,21 +2494,21 @@
         <v>10</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B21" s="7">
         <v>20</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="D21" s="4" t="s">
         <v>17</v>
@@ -2523,27 +2523,27 @@
         <v>10</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B22" s="7">
         <v>21</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="D22" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F22" s="1" t="s">
         <v>19</v>
@@ -2552,21 +2552,21 @@
         <v>10</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="B23" s="7">
         <v>22</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="D23" s="4" t="s">
         <v>17</v>
@@ -2581,27 +2581,27 @@
         <v>10</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="B24" s="7">
         <v>23</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="D24" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F24" s="1" t="s">
         <v>19</v>
@@ -2610,21 +2610,21 @@
         <v>10</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="B25" s="7">
         <v>24</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>17</v>
@@ -2639,27 +2639,27 @@
         <v>10</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="B26" s="7">
         <v>25</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="D26" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F26" s="1" t="s">
         <v>19</v>
@@ -2668,21 +2668,21 @@
         <v>10</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B27" s="7">
         <v>26</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>17</v>
@@ -2697,21 +2697,21 @@
         <v>10</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B28" s="7">
         <v>27</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>17</v>
@@ -2726,21 +2726,21 @@
         <v>10</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="B29" s="7">
         <v>28</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="D29" s="4" t="s">
         <v>17</v>
@@ -2755,21 +2755,21 @@
         <v>10</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="B30" s="7">
         <v>29</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="D30" s="4" t="s">
         <v>17</v>
@@ -2784,27 +2784,27 @@
         <v>10</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="B31" s="7">
         <v>30</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="D31" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F31" s="1" t="s">
         <v>19</v>
@@ -2813,27 +2813,27 @@
         <v>10</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="B32" s="7">
         <v>31</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D32" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F32" s="1" t="s">
         <v>19</v>
@@ -2842,21 +2842,21 @@
         <v>10</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="7">
         <v>32</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D33" s="4" t="s">
         <v>17</v>
@@ -2871,21 +2871,21 @@
         <v>10</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B34" s="7">
         <v>33</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>17</v>
@@ -2900,27 +2900,27 @@
         <v>10</v>
       </c>
       <c r="H34" s="3" t="s">
-        <v>20</v>
+        <v>485</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="B35" s="7">
         <v>34</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="D35" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="F35" s="1" t="s">
         <v>19</v>
@@ -2929,39 +2929,39 @@
         <v>10</v>
       </c>
       <c r="H35" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="8" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B36" s="1">
         <v>35</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="D36" s="4" t="s">
         <v>17</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>10</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>20</v>
+        <v>278</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2970,15 +2970,12 @@
       <sortCondition ref="B1"/>
     </sortState>
   </autoFilter>
-  <dataValidations count="6">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="F2:F36" xr:uid="{06D99139-2FA3-4AFB-B1C3-3BEE2A9AAD12}">
       <formula1>ParamValues6</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="G2:G36" xr:uid="{1151C22F-EEEC-41FC-9B99-4E6AF0576CD2}">
       <formula1>ParamValues7</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="H2:H36" xr:uid="{616A26CB-D9F9-4D1C-BA1B-E708E2CBE0E9}">
-      <formula1>ParamValues8</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="The inserted value is not valid. Please select a value from the dropdown list" sqref="I2:I36" xr:uid="{B1E7E558-C3C7-40E8-8539-FFB9D8F8545E}">
       <formula1>ParamValues13</formula1>
@@ -3018,13 +3015,13 @@
         <v>17</v>
       </c>
       <c r="F1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="G1" t="s">
         <v>10</v>
       </c>
       <c r="H1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="I1" t="s">
         <v>12</v>
@@ -3044,13 +3041,13 @@
         <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H2" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="I2" t="s">
         <v>13</v>
@@ -3062,70 +3059,70 @@
         <v>13</v>
       </c>
       <c r="M2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="H3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="H5" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="H6" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="4:13" x14ac:dyDescent="0.25">
       <c r="D7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F7" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="H7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F8" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="9" spans="4:13" x14ac:dyDescent="0.25">
@@ -3133,7 +3130,7 @@
         <v>8</v>
       </c>
       <c r="H9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="10" spans="4:13" x14ac:dyDescent="0.25">
@@ -3141,263 +3138,263 @@
         <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="11" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F11" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H11" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H12" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="13" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H13" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="14" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H14" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="15" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H15" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" spans="4:13" x14ac:dyDescent="0.25">
       <c r="F16" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H16" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="17" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H17" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="18" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F18" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="H18" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F19" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="H19" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="20" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H20" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="21" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F21" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H21" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="22" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F22" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H22" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F23" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="H23" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="24" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F24" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="25" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F25" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H25" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="26" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F26" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H26" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="27" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F27" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H27" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="28" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F28" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H28" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F29" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H29" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F30" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H30" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="31" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F31" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H31" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="32" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F32" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H32" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F33" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H33" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="34" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F34" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H34" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="35" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F35" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H35" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="36" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F36" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H36" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="37" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F37" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H37" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="38" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F38" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H38" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="39" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F39" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H39" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="40" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F40" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H40" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="41" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H41" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="42" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F42" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H42" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="43" spans="6:8" x14ac:dyDescent="0.25">
@@ -3405,15 +3402,15 @@
         <v>18</v>
       </c>
       <c r="H43" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="44" spans="6:8" x14ac:dyDescent="0.25">
       <c r="F44" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H44" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="45" spans="6:8" x14ac:dyDescent="0.25">
@@ -3421,87 +3418,87 @@
         <v>6</v>
       </c>
       <c r="H45" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="46" spans="6:8" x14ac:dyDescent="0.25">
       <c r="H46" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="47" spans="6:8" x14ac:dyDescent="0.25">
       <c r="H47" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="48" spans="6:8" x14ac:dyDescent="0.25">
       <c r="H48" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="49" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H49" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="50" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H50" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="51" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H51" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="52" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H52" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="53" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H53" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="54" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H54" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="55" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H55" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="56" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H56" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="57" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H57" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="58" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H58" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="59" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H59" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="60" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H60" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="61" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H61" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="62" spans="8:8" x14ac:dyDescent="0.25">
@@ -3511,732 +3508,732 @@
     </row>
     <row r="63" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H63" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="64" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H64" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="65" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H65" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="66" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H66" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="67" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H67" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="68" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H68" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="69" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H69" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="70" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H70" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="71" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H71" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="72" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H72" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="73" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H73" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="74" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H74" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="75" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H75" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="76" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H76" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="77" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H77" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="78" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H78" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="79" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H79" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="80" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H80" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="81" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H81" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="82" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H82" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="83" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H83" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="84" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H84" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="85" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H85" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="86" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H86" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="87" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H87" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="88" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H88" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="89" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H89" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="90" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H90" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="91" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H91" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="92" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H92" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="93" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H93" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="94" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H94" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="95" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H95" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="96" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H96" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="97" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H97" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="98" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H98" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="99" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H99" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="100" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H100" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="101" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H101" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="102" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H102" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="103" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H103" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="104" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H104" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="105" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H105" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="106" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H106" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="107" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H107" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="108" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H108" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="109" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H109" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="110" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H110" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="111" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H111" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
     <row r="112" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H112" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="113" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H113" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="114" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H114" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="115" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H115" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="116" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H116" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="117" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H117" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="118" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H118" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="119" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H119" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="120" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H120" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="121" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H121" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="122" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H122" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="123" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H123" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="124" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H124" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="125" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H125" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="126" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H126" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="127" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H127" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="128" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H128" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="129" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H129" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="130" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H130" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="131" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H131" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="132" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H132" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="133" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H133" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="134" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H134" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="135" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H135" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="136" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H136" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="137" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H137" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="138" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H138" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="139" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H139" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="140" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H140" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
     </row>
     <row r="141" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H141" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
     </row>
     <row r="142" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H142" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="143" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H143" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="144" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H144" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="145" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H145" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
     </row>
     <row r="146" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H146" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="147" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H147" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
     </row>
     <row r="148" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H148" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
     </row>
     <row r="149" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H149" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
     </row>
     <row r="150" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H150" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
     </row>
     <row r="151" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H151" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
     </row>
     <row r="152" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H152" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
     </row>
     <row r="153" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H153" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="154" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H154" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="155" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H155" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="156" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H156" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="157" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H157" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="158" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H158" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="159" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H159" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="160" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H160" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="161" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H161" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="162" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H162" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="163" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H163" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="164" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H164" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
     <row r="165" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H165" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="166" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H166" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="167" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H167" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="168" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H168" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="169" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H169" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="170" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H170" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="171" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H171" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="172" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H172" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="173" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H173" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="174" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H174" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="175" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H175" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="176" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H176" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="177" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H177" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="178" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H178" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="179" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H179" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="180" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H180" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="181" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H181" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="182" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H182" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="183" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H183" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="184" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H184" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="185" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H185" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="186" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H186" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="187" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H187" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="188" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H188" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="189" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H189" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="190" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H190" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="191" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H191" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="192" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H192" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="193" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H193" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="194" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H194" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="195" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H195" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="196" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H196" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="197" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H197" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="198" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H198" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="199" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H199" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="200" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H200" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="201" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H201" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="202" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H202" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="203" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H203" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="204" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H204" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="205" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H205" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="206" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H206" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="207" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H207" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="208" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H208" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
   </sheetData>
@@ -4253,355 +4250,355 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F3" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D7" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F8" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D9" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F9" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B10" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F10" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F14" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C15" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D15" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B16" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C16" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D16" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C17" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F17" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C18" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B19" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D19" t="s">
         <v>9</v>
@@ -4609,224 +4606,224 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B20" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D20" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B21" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C21" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D21" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C22" t="s">
         <v>18</v>
       </c>
       <c r="D22" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B23" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C23" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D23" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C24" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B25" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C25" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D25" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C26" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D26" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B27" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B28" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B29" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B30" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B31" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B32" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B33" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B34" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -4843,25 +4840,25 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>424</v>
+      </c>
+      <c r="B1" t="s">
         <v>425</v>
-      </c>
-      <c r="B1" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -4871,26 +4868,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1ce2a17a-c0eb-4821-a205-2297eefe49d7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010050F8A84B685D8A4A986E703CF63AF792" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2fa97ab612b8c94963ad725742f68d96">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1ce2a17a-c0eb-4821-a205-2297eefe49d7" xmlns:ns3="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8fd2c164260f873fa57e921d57f91808" ns2:_="" ns3:_="">
     <xsd:import namespace="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
@@ -5097,10 +5074,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="1ce2a17a-c0eb-4821-a205-2297eefe49d7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0ADC3DD0-5BD5-40CE-B970-48D4CA313F4F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0E6C32A-332A-47F8-AA61-6F8F7495A83A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
+    <ds:schemaRef ds:uri="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -5117,20 +5125,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0E6C32A-332A-47F8-AA61-6F8F7495A83A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0ADC3DD0-5BD5-40CE-B970-48D4CA313F4F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="1ce2a17a-c0eb-4821-a205-2297eefe49d7"/>
-    <ds:schemaRef ds:uri="d3d766bc-3a2e-4b05-abf0-3bfac4a5263f"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>